<commit_message>
docs: test report: code review findings, CI fix, seed data change, 305 tests
</commit_message>
<xml_diff>
--- a/Reports/Stage-1-Test-Report.xlsx
+++ b/Reports/Stage-1-Test-Report.xlsx
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Test Results'!C2:C305)</f>
+        <f>COUNTA('Test Results'!C2:C306)</f>
         <v/>
       </c>
     </row>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Results'!E2:E305,"Passed")</f>
+        <f>COUNTIF('Test Results'!E2:E306,"Passed")</f>
         <v/>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Results'!E2:E305,"Failed")</f>
+        <f>COUNTIF('Test Results'!E2:E306,"Failed")</f>
         <v/>
       </c>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Test Results'!E2:E305,"Skipped")</f>
+        <f>COUNTIF('Test Results'!E2:E306,"Skipped")</f>
         <v/>
       </c>
     </row>
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E305"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8810,6 +8810,33 @@
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="4" t="inlineStr">
+        <is>
+          <t>Seeds</t>
+        </is>
+      </c>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>seeds.int.spec.ts</t>
+        </is>
+      </c>
+      <c r="C306" s="4" t="inlineStr">
+        <is>
+          <t>loadSeedData reads the git-ignored list or the committed example, and rejects a broken file</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -8941,7 +8968,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>203 tests.</t>
+          <t>204 tests (203 at the final fix wave; one seed-data test added 27 October).</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -9507,12 +9534,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>NEON_AUTH_BASE_URL and NEON_AUTH_COOKIE_SECRET are not yet added to the KANDO GitHub repository, so CI cannot run the web tests.</t>
+          <t>Optional: without NEON_AUTH_BASE_URL and NEON_AUTH_COOKIE_SECRET the one test against the real Neon Auth is skipped in CI. CI is green without them.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner, optional</t>
         </is>
       </c>
     </row>
@@ -9904,6 +9931,108 @@
       <c r="C27" s="4" t="inlineStr">
         <is>
           <t>South Africa work</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>CI: categories seed test failed on GitHub</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Counted all categories; other spec files leave their own behind in the shared CI database. Counts only the seeded slugs now. Fixed in 67c80bb; CI green since.</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Seed account list out of git (owner request, 27 October)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>The 14 test accounts, their password and made-up profiles were in packages/domain/src/seed/test-users.ts in a public repository. Now read from the git-ignored seed-data/test-users.json; a one-customer-one-provider example file is committed; tests use their own fixture. Fixed in a72cf74. Earlier commits still hold the list: squash-merge PR #2 and delete the branch.</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Code review 27 October (mobile build config), 1 of 6: microphone permission</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>The image-picker plugin added android.permission.RECORD_AUDIO and an iOS microphone text by default; the app never records audio. Plugin option microphonePermission=false, hand-written permissions list removed. Resolved config checked: no microphone entry. Fixed in 27ea70c.</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Code review 27 October, 2 of 6: production API address</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>The production build profile did not pin EXPO_PUBLIC_API_URL, so a local build could bake in a LAN address. Pinned to https://skillweb.space like the preview profile. Fixed in 27ea70c.</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Code review 27 October, 3 to 5 of 6: dead configuration</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Empty ios.infoPlist, the router asyncRoutes block the plugin overwrites, and the empty submit.production placeholder removed. Fixed in 27ea70c.</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Code review 27 October, 6 of 6: README duplication</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Concerns the old skill-web README only (development-build status repeated in two places). Not applicable to KANDO.</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>

</xml_diff>